<commit_message>
Expand company lists (63 total) and regenerate .xlsx spreadsheet
Co-authored-by: PL77239 <PL77239@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Leather_Goods_Wholesalers.xlsx
+++ b/Leather_Goods_Wholesalers.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Leather Goods Wholesalers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leather Goods Wholesalers'!$A$1:$D$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leather Goods Wholesalers'!$A$1:$D$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -716,61 +716,61 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Lithuania</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>UAB Sominta</t>
+          <t>Esquire Lederwaren – Rupp &amp; Ricker GmbH</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>https://sominta.com</t>
+          <t>https://www.esquire-lederwaren.de</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>info@sominta.lt</t>
+          <t>info@esquire-lederwaren.de</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Lithuania</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>UAB Vilga</t>
+          <t>MB Lederwaren-Importe GmbH</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>http://www.vilga.lt</t>
+          <t>https://www.mb-lederwaren.de</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>info@vilga.lt</t>
+          <t>info@mb-lederwaren.de</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Lithuania</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>UAB Arenalis (leather materials)</t>
+          <t>LM-International (Europa) GmbH (Rimbaldi / Woodland)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>https://www.leather.lt</t>
+          <t>https://lmi.de</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
@@ -778,15 +778,19 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Lithuania</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Baltijos odos, MB / Baltic Leather Supply (leather materials)</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr"/>
+          <t>Koffer-Zentrale.de (direct importer)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>https://koffer-zentrale.de</t>
+        </is>
+      </c>
       <c r="D16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
@@ -797,88 +801,96 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Revaris (leather materials)</t>
+          <t>UAB Sominta</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>https://www.revaris.lt</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
+          <t>https://sominta.com</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>info@sominta.lt</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Latvia</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>SIA Mille</t>
+          <t>UAB Vilga</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>https://www.mille.lv</t>
+          <t>http://www.vilga.lt</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>mille@mille.lv</t>
+          <t>info@vilga.lt</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Latvia</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Modes Elementi</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr"/>
-      <c r="D19" s="2" t="inlineStr"/>
+          <t>ANIS, UAB</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.anis.lt</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>info@anis.lt</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Latvia</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>SIA Velplev</t>
+          <t>VIKTODA, UAB</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>https://www.velplev.lv</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>velplev@inbox.lv</t>
-        </is>
-      </c>
+          <t>http://www.viktoda.lt</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Latvia</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Tailor Riga (SIA ALIAS-Z)</t>
+          <t>UAB Arenalis (leather materials)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>https://www.tailorriga.lv</t>
+          <t>https://www.leather.lt</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
@@ -886,35 +898,31 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Latvia</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Eric Lasko Production</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>https://ericlasko.com</t>
-        </is>
-      </c>
+          <t>Baltijos odos, MB / Baltic Leather Supply (leather materials)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Latvia</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Lakolina (directory listing - verify)</t>
+          <t>Revaris (leather materials)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>https://www.exporthub.com/lakolina/</t>
+          <t>https://www.revaris.lt</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
@@ -922,79 +930,75 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Estonia</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Nabo Nahktooted OÜ (Nokian Nahkatuote group)</t>
+          <t>SIA Mille</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>https://nokiannahkatuote.fi</t>
+          <t>https://www.mille.lv</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>nabo@nahkatuote.inet.fi</t>
+          <t>mille@mille.lv</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Estonia</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Bagy OÜ</t>
+          <t>Modes Elementi</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>bettigehrke@gmail.com</t>
-        </is>
-      </c>
+      <c r="D25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Estonia</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Leather World OÜ (leather materials / footwear)</t>
+          <t>SIA Velplev</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>https://leather-world.co</t>
+          <t>https://www.velplev.lv</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>sales@leather-world.co</t>
+          <t>velplev@inbox.lv</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Estonia</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Nakro OÜ (leather materials)</t>
+          <t>Tailor Riga (SIA ALIAS-Z)</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>https://www.nakro.ee</t>
+          <t>https://www.tailorriga.lv</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
@@ -1002,83 +1006,75 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>JUNI EXPORT-IMPORT s.r.o.</t>
+          <t>Eric Lasko Production</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>https://www.juni.cz</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>info@juni.cz</t>
-        </is>
-      </c>
+          <t>https://ericlasko.com</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>PAUL BORDAS FASHION, s.r.o.</t>
+          <t>SB Ādas Dizains (Sandra Birze)</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>https://www.paulbordas.cz</t>
+          <t>https://sbadasdizains.lv</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>info@paulbordas.cz</t>
+          <t>sb@sbadasdizains.lv</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>UNIVARO – leather s.r.o. (UNIVARO Bags)</t>
+          <t>Buduart</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>https://www.univaro.cz</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>info@univaro.cz</t>
-        </is>
-      </c>
+          <t>https://www.buduart.lv</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Gora (gora-velkoobchod)</t>
+          <t>Lakolina (directory listing - verify)</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>https://www.gora-velkoobchod.cz</t>
+          <t>https://www.exporthub.com/lakolina/</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr"/>
@@ -1086,249 +1082,265 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Estonia</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>VEGA-LM (VegaLM)</t>
+          <t>Gasell AS</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>https://www.vegalm.sk</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr"/>
+          <t>https://gasell.ee</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>gasell@gasell.ee</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Estonia</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Max s.r.o. (MAX Original Leather / MaxLeather)</t>
+          <t>Nabo Nahktooted OÜ (Nokian Nahkatuote group)</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>https://maxleather.sk</t>
+          <t>https://nokiannahkatuote.fi</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>max@maxleather.sk</t>
+          <t>nabo@nahkatuote.inet.fi</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Estonia</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>NICOLAUS LEATHER, s.r.o. (leather materials)</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>https://nicolausleather.sk</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr"/>
+          <t>Bagy OÜ</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>bettigehrke@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Estonia</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>BI-KA Bőráru Kft.</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>https://divatnagyker.hu/bi-ka-boraru-kft-bordiszmu-aru-importor-nagykereskedo/</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr"/>
+          <t>Fashion House Eesti OÜ</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>leif.karlsson@meridiangroup.eu</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Estonia</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Skin Bőrdíszmű</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr"/>
+          <t>Stalcom OÜ</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>https://stalcom.ee</t>
+        </is>
+      </c>
       <c r="D36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Estonia</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Synchrony LM (SLM Bőrdíszmű / Bőrdíszműnagyker)</t>
+          <t>Leather World OÜ (leather materials / footwear)</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>https://bordiszmunagyker.hu</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr"/>
+          <t>https://leather-world.co</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>sales@leather-world.co</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Estonia</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Kadro Bőrdíszmű Nagykereskedés</t>
+          <t>Nakro OÜ (leather materials)</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>https://kadro.hu</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>info@kadro.hu</t>
-        </is>
-      </c>
+          <t>https://www.nakro.ee</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Top Bag 2000 Kft. (Karen)</t>
+          <t>JUNI EXPORT-IMPORT s.r.o.</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>https://karennagyker.hu</t>
+          <t>https://www.juni.cz</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>info@karen.hu</t>
+          <t>info@juni.cz</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Axelsen &amp; Søn ApS (Montana / Treats)</t>
+          <t>PAUL BORDAS FASHION, s.r.o.</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>https://axelsenson.com</t>
+          <t>https://www.paulbordas.cz</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>info@axelsenson.com</t>
+          <t>info@paulbordas.cz</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Uni-Leather ApS</t>
+          <t>UNIVARO – leather s.r.o. (UNIVARO Bags)</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>https://uni-leather.dk</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr"/>
+          <t>https://www.univaro.cz</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>info@univaro.cz</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Adax A/S</t>
+          <t>SEGALI</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>https://adax.dk</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr"/>
+          <t>https://www.segali.cz</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>velkoobchod@segali.cz</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Markberg</t>
+          <t>Kožená galanterie GaToLi (Libor Tomáš)</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>https://markberg.dk</t>
+          <t>https://e-jola.webnode.cz</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>salessupport@markberg.com</t>
+          <t>libor.tomas@avonet.cz</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Still Nordic</t>
+          <t>Gora (gora-velkoobchod)</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>https://stillnordic.dk</t>
+          <t>https://www.gora-velkoobchod.cz</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr"/>
@@ -1336,45 +1348,405 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>SIPO Trading K/S (leather / skins)</t>
+          <t>VEGA-LM (VegaLM)</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>https://sipo.dk</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr"/>
+          <t>https://www.vegalm.sk</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>vega@vegalm.sk</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
+          <t>Slovakia</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Arwel, s.r.o.</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.arwel.sk</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Slovakia</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Max s.r.o. (MAX Original Leather / MaxLeather)</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>https://maxleather.sk</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>max@maxleather.sk</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Slovakia</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>NICOLAUS LEATHER, s.r.o. (leather materials)</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>https://nicolausleather.sk</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>BI-KA Bőráru Kft.</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>https://bikabor.hu</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>bikabor@bikabor.hu</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Skin Bőrdíszmű Nagykereskedés (Skintaska)</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>https://skintaska.hu</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Synchrony LM (SLM Bőrdíszmű / Bőrdíszműnagyker)</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>https://bordiszmunagyker.hu</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>info@bordiszmunagyker.hu</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Kadro Bőrdíszmű Nagykereskedés</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>https://kadro.hu</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>info@kadro.hu</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Top Bag 2000 Kft. (Karen)</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>https://karennagyker.hu</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>info@karen.hu</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Zolferex Kft. (Nettáska)</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>https://www.nettaska.hu</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>info@zolferex.hu</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Farkas Bőrdíszmű</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>https://farkasbordiszmu.hu</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
           <t>Denmark</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Axelsen &amp; Søn ApS (Montana / Treats)</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>https://axelsenson.com</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>info@axelsenson.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Uni-Leather ApS</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>https://uni-leather.dk</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Adax A/S</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>https://adax.dk</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Markberg</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>https://markberg.dk</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>salessupport@markberg.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Still Nordic</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>https://stillnordic.dk</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>dbramante1928</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>https://www.dbramante1928.com</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Depeche (Depeche Denmark)</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>https://www.depeche.dk</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>SIPO Trading K/S (leather / skins)</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>https://sipo.dk</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>Sicadan (leather materials)</t>
         </is>
       </c>
-      <c r="C46" s="3" t="inlineStr">
+      <c r="C64" s="3" t="inlineStr">
         <is>
           <t>https://www.sicadan.dk</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr">
+      <c r="D64" s="3" t="inlineStr">
         <is>
           <t>info@sicadan.dk</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D46"/>
+  <autoFilter ref="A1:D64"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
@@ -1400,47 +1772,77 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId95"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Verify companies by fit for selling Indian leather goods; add Fit classification, Priority targets sheet, VERIFICATION.md
Co-authored-by: PL77239 <PL77239@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Leather_Goods_Wholesalers.xlsx
+++ b/Leather_Goods_Wholesalers.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Leather Goods Wholesalers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="All companies" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Priority targets" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leather Goods Wholesalers'!$A$1:$D$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All companies'!$A$1:$F$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Priority targets'!$A$1:$F$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37,7 +39,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +49,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -86,6 +103,18 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -452,13 +481,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,6 +513,16 @@
           <t>E-mail</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Business type</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Fit for buying Indian leather goods</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -504,6 +545,16 @@
           <t>info@impex-lederwaren.de</t>
         </is>
       </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Importer &amp; wholesaler of small leather goods/bags</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -526,6 +577,16 @@
           <t>hmtlederwaren@t-online.de</t>
         </is>
       </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Importer &amp; wholesaler (imports from factories)</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -548,6 +609,16 @@
           <t>info@apc-ncc.de</t>
         </is>
       </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>B2B wholesaler (own brands sourced abroad)</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -570,6 +641,16 @@
           <t>bertoni-grosshandel@web.de</t>
         </is>
       </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>B2B wholesaler of bags/accessories</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -579,15 +660,29 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Branco Lederwaren (Sommer &amp; Grubba GbR)</t>
+          <t>DEIMOS Lederwaren GmbH</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>https://www.branco-lederwaren.de</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
+          <t>https://deimosfashion.com</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>info@deimosfashion.com</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler / cash &amp; carry + private label</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -597,17 +692,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>DEIMOS Lederwaren GmbH</t>
+          <t>CLM Lederwaren GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>https://deimosfashion.com</t>
+          <t>https://clm-shop.de</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>info@deimosfashion.com</t>
+          <t>info@clm-shop.de</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler (brand distribution)</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
         </is>
       </c>
     </row>
@@ -619,17 +724,27 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>CLM Lederwaren GmbH &amp; Co. KG</t>
+          <t>Greenburry (bags for living GmbH)</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>https://clm-shop.de</t>
+          <t>https://www.greenburry.de</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>info@clm-shop.de</t>
+          <t>info@bagsforliving.de</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Brand/importer - already sources finished goods from India &amp; Europe</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
         </is>
       </c>
     </row>
@@ -641,15 +756,29 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Venetto</t>
+          <t>MB Lederwaren-Importe GmbH</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>https://venetto.de</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
+          <t>https://www.mb-lederwaren.de</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>info@mb-lederwaren.de</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Wholesale importer of leather goods/luggage</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -659,17 +788,23 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PICARD Lederwaren GmbH &amp; Co. KG</t>
+          <t>LM-International (Europa) GmbH</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>https://picard-fashion.com</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>tf@picard-fashion.com</t>
+          <t>https://lmi.de</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Importer &amp; wholesaler (imports all articles itself)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
         </is>
       </c>
     </row>
@@ -681,17 +816,23 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Braun Büffel (Braun GmbH &amp; Co. KG)</t>
+          <t>Koffer-Zentrale.de</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>https://braun-bueffel.com</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>info@braun-bueffel.com</t>
+          <t>https://koffer-zentrale.de</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Direct importer / B2B wholesaler (dealers only)</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
         </is>
       </c>
     </row>
@@ -703,15 +844,25 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Greenburry</t>
+          <t>Branco Lederwaren (Sommer &amp; Grubba GbR)</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>https://www.greenburry.de</t>
+          <t>https://www.branco-lederwaren.de</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Own production + private label (manufacturer)</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -721,17 +872,27 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Esquire Lederwaren – Rupp &amp; Ricker GmbH</t>
+          <t>PICARD Lederwaren GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>https://www.esquire-lederwaren.de</t>
+          <t>https://picard-fashion.com</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>info@esquire-lederwaren.de</t>
+          <t>tf@picard-fashion.com</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Manufacturer/brand (own production EU) + private label</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
         </is>
       </c>
     </row>
@@ -743,17 +904,23 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>MB Lederwaren-Importe GmbH</t>
+          <t>Venetto</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>https://www.mb-lederwaren.de</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>info@mb-lederwaren.de</t>
+          <t>https://venetto.de</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Own manufacturer 'Made in Germany'</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
         </is>
       </c>
     </row>
@@ -765,15 +932,29 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>LM-International (Europa) GmbH (Rimbaldi / Woodland)</t>
+          <t>Braun Büffel (Braun GmbH &amp; Co. KG)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>https://lmi.de</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
+          <t>https://braun-bueffel.com</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>info@braun-bueffel.com</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Own manufacturer 'Made in Germany' (premium)</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -783,15 +964,29 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Koffer-Zentrale.de (direct importer)</t>
+          <t>Esquire Lederwaren – Rupp &amp; Ricker GmbH</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>https://koffer-zentrale.de</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
+          <t>https://www.esquire-lederwaren.de</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>info@esquire-lederwaren.de</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Own manufacturer/brand (own factory, own patents)</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -801,17 +996,27 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>UAB Sominta</t>
+          <t>ANIS, UAB</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>https://sominta.com</t>
+          <t>https://www.anis.lt</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>info@sominta.lt</t>
+          <t>info@anis.lt</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Distributor/importer of brands + retail (wholesale &amp; retail)</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
         </is>
       </c>
     </row>
@@ -823,17 +1028,27 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>UAB Vilga</t>
+          <t>UAB Sominta</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>http://www.vilga.lt</t>
+          <t>https://sominta.com</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>info@vilga.lt</t>
+          <t>info@sominta.lt</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Own manufacturer (handbags) + contract mfr</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
         </is>
       </c>
     </row>
@@ -845,17 +1060,27 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>ANIS, UAB</t>
+          <t>UAB Vilga</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>https://www.anis.lt</t>
+          <t>http://www.vilga.lt</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>info@anis.lt</t>
+          <t>info@vilga.lt</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Own manufacturer (natural leather goods)</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
         </is>
       </c>
     </row>
@@ -876,6 +1101,16 @@
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Own manufacturer + trade</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -885,7 +1120,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>UAB Arenalis (leather materials)</t>
+          <t>UAB Arenalis</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -894,6 +1129,16 @@
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Leather materials / hides &amp; fittings</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -903,11 +1148,21 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Baltijos odos, MB / Baltic Leather Supply (leather materials)</t>
+          <t>Baltijos odos, MB / Baltic Leather Supply</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Leather materials / hides &amp; fittings</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -917,7 +1172,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Revaris (leather materials)</t>
+          <t>Revaris</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -926,6 +1181,16 @@
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Leather materials (natural &amp; artificial)</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -935,17 +1200,19 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>SIA Mille</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mille.lv</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>mille@mille.lv</t>
+          <t>Modes Elementi</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Distributor/wholesaler of branded accessories (stock)</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
         </is>
       </c>
     </row>
@@ -957,11 +1224,29 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Modes Elementi</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr"/>
-      <c r="D25" s="2" t="inlineStr"/>
+          <t>SIA Mille</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mille.lv</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>mille@mille.lv</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Own manufacturer (produces for brands) / OEM</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -984,6 +1269,16 @@
           <t>velplev@inbox.lv</t>
         </is>
       </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Own manufacturer (bag production)</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1002,6 +1297,16 @@
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Own manufacturer / artisan</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1020,6 +1325,16 @@
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Artisan manufacturer (no outsourcing, no mass production)</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1042,6 +1357,16 @@
           <t>sb@sbadasdizains.lv</t>
         </is>
       </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Artisan handmade manufacturer</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1060,6 +1385,16 @@
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Own-design brand / own workshop</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1069,7 +1404,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Lakolina (directory listing - verify)</t>
+          <t>Lakolina</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -1078,6 +1413,16 @@
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Directory listing; appears own-make - unverified</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1100,6 +1445,16 @@
           <t>gasell@gasell.ee</t>
         </is>
       </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler &amp; importer (maaletooja) of bags/accessories</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1109,7 +1464,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Nabo Nahktooted OÜ (Nokian Nahkatuote group)</t>
+          <t>Nabo Nahktooted OÜ</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -1120,6 +1475,16 @@
       <c r="D33" s="3" t="inlineStr">
         <is>
           <t>nabo@nahkatuote.inet.fi</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Importer + manufacturer (imports finished bags/wallets)</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
         </is>
       </c>
     </row>
@@ -1140,6 +1505,16 @@
           <t>bettigehrke@gmail.com</t>
         </is>
       </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Wholesale agent for leather goods</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1158,6 +1533,16 @@
           <t>leif.karlsson@meridiangroup.eu</t>
         </is>
       </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Wholesale agent for leather goods</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1176,6 +1561,16 @@
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Custom leather goods producer + wholesale</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1185,7 +1580,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Leather World OÜ (leather materials / footwear)</t>
+          <t>Leather World OÜ</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -1196,6 +1591,16 @@
       <c r="D37" s="3" t="inlineStr">
         <is>
           <t>sales@leather-world.co</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Leather materials / footwear distribution</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1612,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Nakro OÜ (leather materials)</t>
+          <t>Nakro OÜ</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -1216,6 +1621,16 @@
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Leather materials / tannery</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1238,6 +1653,16 @@
           <t>info@juni.cz</t>
         </is>
       </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Importer &amp; wholesaler of leather goods</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1260,6 +1685,16 @@
           <t>info@paulbordas.cz</t>
         </is>
       </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Distributor/importer (represents foreign brands)</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1269,7 +1704,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>UNIVARO – leather s.r.o. (UNIVARO Bags)</t>
+          <t>UNIVARO – leather s.r.o.</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -1280,6 +1715,16 @@
       <c r="D41" s="3" t="inlineStr">
         <is>
           <t>info@univaro.cz</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Exclusive importer/distributor of brands</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
         </is>
       </c>
     </row>
@@ -1291,17 +1736,27 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>SEGALI</t>
+          <t>Kožená galanterie GaToLi (Libor Tomáš)</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>https://www.segali.cz</t>
+          <t>https://e-jola.webnode.cz</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>velkoobchod@segali.cz</t>
+          <t>libor.tomas@avonet.cz</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler/distributor of leather goods</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
         </is>
       </c>
     </row>
@@ -1313,17 +1768,23 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Kožená galanterie GaToLi (Libor Tomáš)</t>
+          <t>Gora (gora-velkoobchod)</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>https://e-jola.webnode.cz</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>libor.tomas@avonet.cz</t>
+          <t>https://www.gora-velkoobchod.cz</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr"/>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler of leather goods (verify)</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
         </is>
       </c>
     </row>
@@ -1335,35 +1796,55 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Gora (gora-velkoobchod)</t>
+          <t>Karoly (Letohrad)</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>https://www.gora-velkoobchod.cz</t>
+          <t>https://www.firmy.cz/detail/12856470-karoly-letohrad-cervena.html</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler &amp; importer of leather goods</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>VEGA-LM (VegaLM)</t>
+          <t>SEGALI</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>https://www.vegalm.sk</t>
+          <t>https://www.segali.cz</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>vega@vegalm.sk</t>
+          <t>velkoobchod@segali.cz</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Own manufacturer + wholesale / private label</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
         </is>
       </c>
     </row>
@@ -1375,15 +1856,29 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Arwel, s.r.o.</t>
+          <t>Max s.r.o. (MAX Original Leather)</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>https://www.arwel.sk</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr"/>
+          <t>https://maxleather.sk</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>max@maxleather.sk</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>Importer of Italian leather goods + wholesale</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1393,17 +1888,27 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Max s.r.o. (MAX Original Leather / MaxLeather)</t>
+          <t>VEGA-LM (VegaLM)</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>https://maxleather.sk</t>
+          <t>https://www.vegalm.sk</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>max@maxleather.sk</t>
+          <t>vega@vegalm.sk</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Own manufacturer + wholesale/retail</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
         </is>
       </c>
     </row>
@@ -1415,35 +1920,51 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>NICOLAUS LEATHER, s.r.o. (leather materials)</t>
+          <t>Arwel, s.r.o.</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>https://nicolausleather.sk</t>
+          <t>https://www.arwel.sk</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>Own manufacturer + wholesale</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>BI-KA Bőráru Kft.</t>
+          <t>NICOLAUS LEATHER, s.r.o.</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>https://bikabor.hu</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>bikabor@bikabor.hu</t>
+          <t>https://nicolausleather.sk</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr"/>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Leather materials (bovine leather production)</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
         </is>
       </c>
     </row>
@@ -1455,15 +1976,25 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Skin Bőrdíszmű Nagykereskedés (Skintaska)</t>
+          <t>Farkas Bőrdíszmű</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>https://skintaska.hu</t>
+          <t>https://farkasbordiszmu.hu</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>Importer/wholesaler - imports directly from India, China, Poland, Italy, Germany</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1473,17 +2004,27 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Synchrony LM (SLM Bőrdíszmű / Bőrdíszműnagyker)</t>
+          <t>BI-KA Bőráru Kft.</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>https://bordiszmunagyker.hu</t>
+          <t>https://bikabor.hu</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>info@bordiszmunagyker.hu</t>
+          <t>bikabor@bikabor.hu</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>Importer &amp; wholesaler (imports from Italy etc.)</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
         </is>
       </c>
     </row>
@@ -1495,17 +2036,23 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Kadro Bőrdíszmű Nagykereskedés</t>
+          <t>Skin Bőrdíszmű Nagykereskedés (Skintaska)</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>https://kadro.hu</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>info@kadro.hu</t>
+          <t>https://skintaska.hu</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler/importer (Hungarian &amp; imported goods)</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
         </is>
       </c>
     </row>
@@ -1517,17 +2064,27 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Top Bag 2000 Kft. (Karen)</t>
+          <t>Synchrony LM (SLM / Bőrdíszműnagyker)</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>https://karennagyker.hu</t>
+          <t>https://bordiszmunagyker.hu</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>info@karen.hu</t>
+          <t>info@bordiszmunagyker.hu</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler of leather goods</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
         </is>
       </c>
     </row>
@@ -1539,17 +2096,27 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Zolferex Kft. (Nettáska)</t>
+          <t>Kadro Bőrdíszmű Nagykereskedés</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>https://www.nettaska.hu</t>
+          <t>https://kadro.hu</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>info@zolferex.hu</t>
+          <t>info@kadro.hu</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler (sells to resellers only)</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
         </is>
       </c>
     </row>
@@ -1561,35 +2128,59 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Farkas Bőrdíszmű</t>
+          <t>Top Bag 2000 Kft. (Karen)</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>https://farkasbordiszmu.hu</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr"/>
+          <t>https://karennagyker.hu</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>info@karen.hu</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler/distributor of bag brands</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Hungary</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Axelsen &amp; Søn ApS (Montana / Treats)</t>
+          <t>Zolferex Kft. (Nettáska)</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>https://axelsenson.com</t>
+          <t>https://www.nettaska.hu</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>info@axelsenson.com</t>
+          <t>info@zolferex.hu</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>Importer/distributor (exclusive importer of EU brands)</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
         </is>
       </c>
     </row>
@@ -1610,6 +2201,16 @@
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr"/>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>Wholesale; makes own leather goods + imports shoes</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1619,15 +2220,29 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Adax A/S</t>
+          <t>Axelsen &amp; Søn ApS (Montana/Treats)</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>https://adax.dk</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr"/>
+          <t>https://axelsenson.com</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>info@axelsenson.com</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>Manufacturer + B2B custom/personalized</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -1637,17 +2252,23 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Markberg</t>
+          <t>Adax A/S</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>https://markberg.dk</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>salessupport@markberg.com</t>
+          <t>https://adax.dk</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr"/>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>Own-design brand - already produces in India (OEM prospect)</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
         </is>
       </c>
     </row>
@@ -1659,15 +2280,29 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Still Nordic</t>
+          <t>Markberg</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>https://stillnordic.dk</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr"/>
+          <t>https://markberg.dk</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>salessupport@markberg.com</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>Own-design brand - contract mfr worldwide (OEM prospect)</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -1677,15 +2312,25 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>dbramante1928</t>
+          <t>Still Nordic</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>https://www.dbramante1928.com</t>
+          <t>https://stillnordic.dk</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr"/>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>Own-design brand (OEM prospect)</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -1695,15 +2340,25 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Depeche (Depeche Denmark)</t>
+          <t>dbramante1928</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>https://www.depeche.dk</t>
+          <t>https://www.dbramante1928.com</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr"/>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>Own-design brand (cases/bags)</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -1713,15 +2368,25 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>SIPO Trading K/S (leather / skins)</t>
+          <t>Depeche (Depeche Denmark)</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>https://sipo.dk</t>
+          <t>https://www.depeche.dk</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr"/>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>Own-design brand</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>Maybe - own production or own-design brand (only if you offer OEM / private label)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -1731,22 +2396,60 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Sicadan (leather materials)</t>
+          <t>SIPO Trading K/S</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
+          <t>https://sipo.dk</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr"/>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>Leather / skins / fur materials</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Sicadan</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
           <t>https://www.sicadan.dk</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr">
+      <c r="D65" s="3" t="inlineStr">
         <is>
           <t>info@sicadan.dk</t>
         </is>
       </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>Leather materials for manufacturers</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>No - materials/hides/footwear supplier or artisan own-make / not a finished-goods buyer</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D64"/>
+  <autoFilter ref="A1:F65"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
@@ -1757,92 +2460,1121 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId97"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Company Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>WWW</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>E-mail</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Business type</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Fit for buying Indian leather goods</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>iMPEX Lederwaren Import-Export GmbH</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.impex-lederwaren.de</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>info@impex-lederwaren.de</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Importer &amp; wholesaler of small leather goods/bags</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>HMT Lederwaren Import GmbH</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>https://hmtlederwaren.de</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>hmtlederwaren@t-online.de</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Importer &amp; wholesaler (imports from factories)</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>APC-NCC Lederwaren</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>https://apc-ncc.de</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>info@apc-ncc.de</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>B2B wholesaler (own brands sourced abroad)</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Bertoni Großhandel</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>https://bertoni-grosshandel.de</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>bertoni-grosshandel@web.de</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>B2B wholesaler of bags/accessories</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>DEIMOS Lederwaren GmbH</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>https://deimosfashion.com</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>info@deimosfashion.com</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler / cash &amp; carry + private label</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>CLM Lederwaren GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>https://clm-shop.de</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>info@clm-shop.de</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler (brand distribution)</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Greenburry (bags for living GmbH)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.greenburry.de</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>info@bagsforliving.de</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Brand/importer - already sources finished goods from India &amp; Europe</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>MB Lederwaren-Importe GmbH</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mb-lederwaren.de</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>info@mb-lederwaren.de</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Wholesale importer of leather goods/luggage</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>LM-International (Europa) GmbH</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>https://lmi.de</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Importer &amp; wholesaler (imports all articles itself)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Koffer-Zentrale.de</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>https://koffer-zentrale.de</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Direct importer / B2B wholesaler (dealers only)</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Lithuania</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>ANIS, UAB</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.anis.lt</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>info@anis.lt</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Distributor/importer of brands + retail (wholesale &amp; retail)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Latvia</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Modes Elementi</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Distributor/wholesaler of branded accessories (stock)</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Estonia</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Gasell AS</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>https://gasell.ee</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>gasell@gasell.ee</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler &amp; importer (maaletooja) of bags/accessories</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Estonia</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Nabo Nahktooted OÜ</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>https://nokiannahkatuote.fi</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>nabo@nahkatuote.inet.fi</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Importer + manufacturer (imports finished bags/wallets)</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Estonia</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Bagy OÜ</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>bettigehrke@gmail.com</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Wholesale agent for leather goods</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Estonia</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Fashion House Eesti OÜ</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>leif.karlsson@meridiangroup.eu</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Wholesale agent for leather goods</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>JUNI EXPORT-IMPORT s.r.o.</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.juni.cz</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>info@juni.cz</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Importer &amp; wholesaler of leather goods</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>PAUL BORDAS FASHION, s.r.o.</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.paulbordas.cz</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>info@paulbordas.cz</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Distributor/importer (represents foreign brands)</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>UNIVARO – leather s.r.o.</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.univaro.cz</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>info@univaro.cz</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Exclusive importer/distributor of brands</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Kožená galanterie GaToLi (Libor Tomáš)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>https://e-jola.webnode.cz</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>libor.tomas@avonet.cz</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler/distributor of leather goods</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Gora (gora-velkoobchod)</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.gora-velkoobchod.cz</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler of leather goods (verify)</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Karoly (Letohrad)</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmy.cz/detail/12856470-karoly-letohrad-cervena.html</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler &amp; importer of leather goods</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Slovakia</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Max s.r.o. (MAX Original Leather)</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>https://maxleather.sk</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>max@maxleather.sk</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Importer of Italian leather goods + wholesale</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Farkas Bőrdíszmű</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>https://farkasbordiszmu.hu</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Importer/wholesaler - imports directly from India, China, Poland, Italy, Germany</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>BI-KA Bőráru Kft.</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>https://bikabor.hu</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>bikabor@bikabor.hu</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Importer &amp; wholesaler (imports from Italy etc.)</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Skin Bőrdíszmű Nagykereskedés (Skintaska)</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>https://skintaska.hu</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler/importer (Hungarian &amp; imported goods)</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Synchrony LM (SLM / Bőrdíszműnagyker)</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>https://bordiszmunagyker.hu</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>info@bordiszmunagyker.hu</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler of leather goods</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Kadro Bőrdíszmű Nagykereskedés</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>https://kadro.hu</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>info@kadro.hu</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler (sells to resellers only)</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Top Bag 2000 Kft. (Karen)</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>https://karennagyker.hu</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>info@karen.hu</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Wholesaler/distributor of bag brands</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Zolferex Kft. (Nettáska)</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.nettaska.hu</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>info@zolferex.hu</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Importer/distributor (exclusive importer of EU brands)</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Yes - importer / distributor / stock wholesaler (buys finished goods to resell)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F31"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>